<commit_message>
Update Zero2Sudo opportunity tracker and check status
</commit_message>
<xml_diff>
--- a/Zero2Sudo_Opportunity_Tracker.xlsx
+++ b/Zero2Sudo_Opportunity_Tracker.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Opportunities'!$A$1:$R$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Opportunities'!$A$1:$R$51</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R41"/>
+  <dimension ref="A1:R51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4353,8 +4353,907 @@
       </c>
       <c r="R41" s="3" t="inlineStr"/>
     </row>
+    <row r="42" ht="45" customHeight="1">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>314f5c90e2eca63ec5e4</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-18T03:55:59.132604+00:00</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-17T14:48:23+00:00</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>NVIDIA Ignite Internship releases 10/5</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr"/>
+      <c r="H42" s="3" t="inlineStr"/>
+      <c r="I42" s="3" t="inlineStr"/>
+      <c r="J42" s="3" t="inlineStr"/>
+      <c r="K42" s="4" t="inlineStr">
+        <is>
+          <t>https://scontent-dfw5-1.cdninstagram.com/v/t51.82787-15/814875022_18087172547678962_8331711395526830193_n.heic?stp=dst-jpg_e35_sh2.08_tt6&amp;_nc_cat=106&amp;ig_cache_key=Mzk4ODI1MDI4MjU4ODMyMjY1NQ%3D%3D.3-ccb7-5&amp;ccb=7-5&amp;_nc_sid=58cdad&amp;efg=eyJ2ZW5jb2RlX3RhZyI6IlNUT1JZLnhwaWRzLjEwODAuc2RyLnJlZ3VsYXJfcGhvdG8uQzMifQ%3D%3D&amp;_nc_ohc=0lQzvtPz4T8Q7kNvwHCmzto&amp;_nc_oc=AdqbHkWTew8g-pvDOcQ7u7I9Zlgvh21KFC16yyZK0sq59Cll0pfbwzqE_5J3idcA5Ag&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=23&amp;se=7&amp;_nc_ht=scontent-dfw5-1.cdninstagram.com&amp;_nc_gid=eHz5TcyW0mp_pt15cJ6WDA&amp;_nc_ss=7e3ba&amp;oh=00_AQJSzB6lC_tMcAuut_QC3HvLF1mZaTfmuN3IGHFQy4ePSQ&amp;oe=6AB29450</t>
+        </is>
+      </c>
+      <c r="L42" s="4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/stories/zero2sudo/</t>
+        </is>
+      </c>
+      <c r="M42" s="3" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="N42" s="3" t="inlineStr">
+        <is>
+          <t>NVIDIA Ignite Internship releases 10/5
+Turn on your notifications for my account!
+Hey there zero2sudo. | remember
+you mentioning that NVIDIA
+Ignite is going to be released in
+early October. | just got an email
+saying It will be on the 5th
+https://scontent-dfw5-1.cdninstagram.com/v/t51.82787-15/814875022_18087172547678962_8331711395526830193_n.heic?stp=dst-jpg_e35_sh2.08_tt6&amp;_nc_cat=106&amp;ig_cache_key=Mzk4ODI1MDI4MjU4ODMyMjY1NQ%3D%3D.3-ccb7-5&amp;ccb=7-5&amp;_nc_sid=58cdad&amp;efg=eyJ2ZW5jb2RlX3RhZyI6IlNUT1JZLnhwaWRzLjEwODAuc2RyLnJlZ3VsYXJfcGhvdG8uQzMifQ%3D%3D&amp;_nc_ohc=0lQzvtPz4T8Q7kNvwHCmzto&amp;_nc_oc=AdqbHkWTew8g-pvDOcQ7u7I9Zlgvh21KFC16yyZK0sq59Cll0pfbwzqE_5J3idcA5Ag&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=23&amp;se=7&amp;_nc_ht=scontent-dfw5-1.cdninstagram.com&amp;_nc_gid=eHz5TcyW0mp_pt15cJ6WDA&amp;_nc_ss=7e3ba&amp;oh=00_AQJSzB6lC_tMcAuut_QC3HvLF1mZaTfmuN3IGHFQy4ePSQ&amp;oe=6AB29450
+https://scontent-dfw5-1.cdninstagram.com/v/t51.82787-15/814875022_18087172547678962_8331711395526830193_n.heic?stp=dst-jpg_e35_s640x640_sh2.08_tt6&amp;_nc_cat=106&amp;ig_cache_key=Mzk4ODI1MDI4MjU4ODMyMjY1NQ%3D%3D.3-ccb7-5&amp;ccb=7-5&amp;_nc_sid=58cdad&amp;efg=eyJ2ZW5jb2RlX3RhZyI6IlNUT1JZLnhwaWRzLjEwODAuc2RyLnJlZ3VsYXJfcGhvdG8uQzMifQ%3D%3D&amp;_nc_ohc=0lQzvtPz4T8Q7kNvwHCmzto&amp;_nc_oc=AdqbHkWTew8g-pvDOcQ7u7I9Zlgvh21KFC16yyZK0sq59Cll0pfbwzqE_5J3idcA5Ag&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=23&amp;_nc_ht=scontent-dfw5-1.cdninstagram.com&amp;_nc_gid=eHz5TcyW0mp_pt15cJ6WDA&amp;_nc_ss=7e3ba&amp;oh=00_AQIhOBjuFed24yHd6OccDaCRbuDP_jK_Fxqa3avKaJPCjQ&amp;oe=6AB29450
+https://scontent-dfw5-2.cdninstagram.com/v/t51.2885-19/361942212_2508526442658147_3130876906989167533_n.jpg?stp=dst-jpg_e0_s150x150_tt6&amp;_nc_cat=100&amp;ig_cache_key=GMTMkhVjOYbTfekIAK0jkHT1G3MrbkULAAAB1501500j-ccb7-5&amp;ccb=7-5&amp;_nc_sid=669407&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDgwLkMzIn0%3D&amp;_nc_ohc=v_28DqPFYsAQ7kNvwEdRcyz&amp;_nc_oc=Adqw8M_x9B-a8shtOG5wRrb9an7G9olGpS9_wQd75NfCA1HGhLaideM0LC7_0tGzj_o&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=24&amp;_nc_ht=scontent-dfw5-2.cdninstagram.com&amp;_nc_ss=7e3ba&amp;oh=00_AQKjZ8LuZIyQWmMhzZRTIIXPovMdv5VlfhbUe2vSoVvRTA&amp;oe=6AB27099</t>
+        </is>
+      </c>
+      <c r="O42" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="P42" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="Q42" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R42" s="3" t="inlineStr"/>
+    </row>
+    <row r="43" ht="45" customHeight="1">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>f76cd1342a4d1945eb27</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-18T03:56:06.101600+00:00</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-17T15:14:38+00:00</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>Microsoft SWE Intern Offer + Process!</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineering</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>Summer 2027</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="inlineStr"/>
+      <c r="J43" s="3" t="inlineStr"/>
+      <c r="K43" s="4" t="inlineStr">
+        <is>
+          <t>https://scontent-dfw5-2.cdninstagram.com/v/t51.82787-15/813634716_18087176735678962_8479740632337180657_n.heic?stp=dst-jpg_e35_sh2.08_tt6&amp;_nc_cat=107&amp;ig_cache_key=Mzk4ODI2MzQ5NDczOTg1NTczOQ%3D%3D.3-ccb7-5&amp;ccb=7-5&amp;_nc_sid=58cdad&amp;efg=eyJ2ZW5jb2RlX3RhZyI6IlNUT1JZLnhwaWRzLjEwODAuc2RyLnJlZ3VsYXJfcGhvdG8uQzMifQ%3D%3D&amp;_nc_ohc=00WHMxCXizYQ7kNvwGQInUv&amp;_nc_oc=AdocJ6NuB8k-AoviUantdlwnmlMeE9r1u24mtpyK6Xw-RIzvM65J_qyjb1OnxhZb1yA&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=23&amp;se=7&amp;_nc_ht=scontent-dfw5-2.cdninstagram.com&amp;_nc_gid=eHz5TcyW0mp_pt15cJ6WDA&amp;_nc_ss=7e3ba&amp;oh=00_AQIWpRoM3bL_hWlAaIG2tdSjAIMZ-Ktp5xgY_ZxExFGVYA&amp;oe=6AB2A380</t>
+        </is>
+      </c>
+      <c r="L43" s="4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/stories/zero2sudo/</t>
+        </is>
+      </c>
+      <c r="M43" s="3" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="N43" s="3" t="inlineStr">
+        <is>
+          <t>Microsoft SWE Intern Offer + Process!
+Intern Summer 2027, applied as
+soon as | saw your story!
+OA was a standard leetcode easy
+and medium similar to what
+everyone else has been saying
+with the second problem having
+that Al assistant
+v
+First interview had some system
+design, leetcode, and general
+trivia
+Ld
+Second interview was purely
+talking about past experiences
+along with some talk about how |
+use Al to code but it was a super
+chill convo, didn’t feel like an
+interview
+https://scontent-dfw5-2.cdninstagram.com/v/t51.82787-15/813634716_18087176735678962_8479740632337180657_n.heic?stp=dst-jpg_e35_sh2.08_tt6&amp;_nc_cat=107&amp;ig_cache_key=Mzk4ODI2MzQ5NDczOTg1NTczOQ%3D%3D.3-ccb7-5&amp;ccb=7-5&amp;_nc_sid=58cdad&amp;efg=eyJ2ZW5jb2RlX3RhZyI6IlNUT1JZLnhwaWRzLjEwODAuc2RyLnJlZ3VsYXJfcGhvdG8uQzMifQ%3D%3D&amp;_nc_ohc=00WHMxCXizYQ7kNvwGQInUv&amp;_nc_oc=AdocJ6NuB8k-AoviUantdlwnmlMeE9r1u24mtpyK6Xw-RIzvM65J_qyjb1OnxhZb1yA&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=23&amp;se=7&amp;_nc_ht=scontent-dfw5-2.cdninstagram.com&amp;_nc_gid=eHz5TcyW0mp_pt15cJ6WDA&amp;_nc_ss=7e3ba&amp;oh=00_AQIWpRoM3bL_hWlAaIG2tdSjAIMZ-Ktp5xgY_ZxExFGVYA&amp;oe=6AB2A380
+https://scontent-dfw5-2.cdninstagram.com/v/t51.82787-15/813634716_18087176735678962_8479740632337180657_n.heic?stp=dst-jpg_e35_s640x640_sh2.08_tt6&amp;_nc_cat=107&amp;ig_cache_key=Mzk4ODI2MzQ5NDczOTg1NTczOQ%3D%3D.3-ccb7-5&amp;ccb=7-5&amp;_nc_sid=58cdad&amp;efg=eyJ2ZW5jb2RlX3RhZyI6IlNUT1JZLnhwaWRzLjEwODAuc2RyLnJlZ3VsYXJfcGhvdG8uQzMifQ%3D%3D&amp;_nc_ohc=00WHMxCXizYQ7kNvwGQInUv&amp;_nc_oc=AdocJ6NuB8k-AoviUantdlwnmlMeE9r1u24mtpyK6Xw-RIzvM65J_qyjb1OnxhZb1yA&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=23&amp;_nc_ht=scontent-dfw5-2.cdninstagram.com&amp;_nc_gid=eHz5TcyW0mp_pt15cJ6WDA&amp;_nc_ss=7e3ba&amp;oh=00_AQINzKgI3MC1sdOucq-eP4llsOaq6g_uuvlLUpsWYlapgA&amp;oe=6AB2A380
+https://scontent-dfw5-2.cdninstagram.com/v/t51.2885-19/361942212_2508526442658147_3130876906989167533_n.jpg?stp=dst-jpg_e0_s150x150_tt6&amp;_nc_cat=100&amp;ig_cache_key=GMTMkhVjOYbTfekIAK0jkHT1G3MrbkULAAAB1501500j-ccb7-5&amp;ccb=7-5&amp;_nc_sid=669407&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDgwLkMzIn0%3D&amp;_nc_ohc=v_28DqPFYsAQ7kNvwEdRcyz&amp;_nc_oc=Adqw8M_x9B-a8shtOG5wRrb9an7G9olGpS9_wQd75NfCA1HGhLaideM0LC7_0tGzj_o&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=24&amp;_nc_ht=scontent-dfw5-2.cdninstagram.com&amp;_nc_ss=7e3ba&amp;oh=00_AQKjZ8LuZIyQWmMhzZRTIIXPovMdv5VlfhbUe2vSoVvRTA&amp;oe=6AB27099</t>
+        </is>
+      </c>
+      <c r="O43" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="P43" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="Q43" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R43" s="3" t="inlineStr"/>
+    </row>
+    <row r="44" ht="45" customHeight="1">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>4bacd493ca4209df0e9b</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-18T03:56:17.935509+00:00</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-17T16:33:16+00:00</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr"/>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>(new grad swe) yet this year?</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>New Grad / Early Career</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineering</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr"/>
+      <c r="I44" s="3" t="inlineStr"/>
+      <c r="J44" s="3" t="inlineStr"/>
+      <c r="K44" s="4" t="inlineStr">
+        <is>
+          <t>https://scontent-dfw5-2.cdninstagram.com/v/t51.82787-15/814453000_18087186893678962_2860711254553635645_n.heic?stp=dst-jpg_e35_sh2.08_tt6&amp;_nc_cat=104&amp;ig_cache_key=Mzk4ODMwMzA3MjYyMDM1NTkyMA%3D%3D.3-ccb7-5&amp;ccb=7-5&amp;_nc_sid=58cdad&amp;efg=eyJ2ZW5jb2RlX3RhZyI6IlNUT1JZLnhwaWRzLjEwODAuc2RyLnJlZ3VsYXJfcGhvdG8uQzMifQ%3D%3D&amp;_nc_ohc=Kqyif5gxD2UQ7kNvwGrQoN-&amp;_nc_oc=AdpXBVwHSn9OBSr59M00r-W0EnYqJyiF_aC1h_Lt4zXKuOptM0oys_UGzBpCeFAZu8Y&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=23&amp;se=7&amp;_nc_ht=scontent-dfw5-2.cdninstagram.com&amp;_nc_gid=eHz5TcyW0mp_pt15cJ6WDA&amp;_nc_ss=7e3ba&amp;oh=00_AQJYpGfIpiX0j3gyufnEUPSwujZF3lp8kRfx2-SfFf2fxw&amp;oe=6AB29044</t>
+        </is>
+      </c>
+      <c r="L44" s="4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/stories/zero2sudo/</t>
+        </is>
+      </c>
+      <c r="M44" s="3" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="N44" s="3" t="inlineStr">
+        <is>
+          <t>More Cap1 TIP offers! Has anyone gotten TDP
+(new grad swe) yet this year?
+Replied to your story
+Yo | got ci TIP cuz of ur story.
+And the info u dropped was
+exactly what the process was
+like.
+Thank you
+~@
+LFG! im so happy when people
+read the stories and highlights
+and get offers ® there's def
+something about high agency ppl
+who consume info and apply it
+properly and landing roles!
+https://scontent-dfw5-2.cdninstagram.com/v/t51.82787-15/814453000_18087186893678962_2860711254553635645_n.heic?stp=dst-jpg_e35_sh2.08_tt6&amp;_nc_cat=104&amp;ig_cache_key=Mzk4ODMwMzA3MjYyMDM1NTkyMA%3D%3D.3-ccb7-5&amp;ccb=7-5&amp;_nc_sid=58cdad&amp;efg=eyJ2ZW5jb2RlX3RhZyI6IlNUT1JZLnhwaWRzLjEwODAuc2RyLnJlZ3VsYXJfcGhvdG8uQzMifQ%3D%3D&amp;_nc_ohc=Kqyif5gxD2UQ7kNvwGrQoN-&amp;_nc_oc=AdpXBVwHSn9OBSr59M00r-W0EnYqJyiF_aC1h_Lt4zXKuOptM0oys_UGzBpCeFAZu8Y&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=23&amp;se=7&amp;_nc_ht=scontent-dfw5-2.cdninstagram.com&amp;_nc_gid=eHz5TcyW0mp_pt15cJ6WDA&amp;_nc_ss=7e3ba&amp;oh=00_AQJYpGfIpiX0j3gyufnEUPSwujZF3lp8kRfx2-SfFf2fxw&amp;oe=6AB29044
+https://scontent-dfw5-2.cdninstagram.com/v/t51.82787-15/814453000_18087186893678962_2860711254553635645_n.heic?stp=dst-jpg_e35_s640x640_sh2.08_tt6&amp;_nc_cat=104&amp;ig_cache_key=Mzk4ODMwMzA3MjYyMDM1NTkyMA%3D%3D.3-ccb7-5&amp;ccb=7-5&amp;_nc_sid=58cdad&amp;efg=eyJ2ZW5jb2RlX3RhZyI6IlNUT1JZLnhwaWRzLjEwODAuc2RyLnJlZ3VsYXJfcGhvdG8uQzMifQ%3D%3D&amp;_nc_ohc=Kqyif5gxD2UQ7kNvwGrQoN-&amp;_nc_oc=AdpXBVwHSn9OBSr59M00r-W0EnYqJyiF_aC1h_Lt4zXKuOptM0oys_UGzBpCeFAZu8Y&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=23&amp;_nc_ht=scontent-dfw5-2.cdninstagram.com&amp;_nc_gid=eHz5TcyW0mp_pt15cJ6WDA&amp;_nc_ss=7e3ba&amp;oh=00_AQKzt6EFQ7rBlpyBBx_IwzIWSM_qcMutuHsAfaFz1Gi8_Q&amp;oe=6AB29044
+https://scontent-dfw5-2.cdninstagram.com/v/t51.2885-19/361942212_2508526442658147_3130876906989167533_n.jpg?stp=dst-jpg_e0_s150x150_tt6&amp;_nc_cat=100&amp;ig_cache_key=GMTMkhVjOYbTfekIAK0jkHT1G3MrbkULAAAB1501500j-ccb7-5&amp;ccb=7-5&amp;_nc_sid=669407&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDgwLkMzIn0%3D&amp;_nc_ohc=v_28DqPFYsAQ7kNvwEdRcyz&amp;_nc_oc=Adqw8M_x9B-a8shtOG5wRrb9an7G9olGpS9_wQd75NfCA1HGhLaideM0LC7_0tGzj_o&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=24&amp;_nc_ht=scontent-dfw5-2.cdninstagram.com&amp;_nc_ss=7e3ba&amp;oh=00_AQKjZ8LuZIyQWmMhzZRTIIXPovMdv5VlfhbUe2vSoVvRTA&amp;oe=6AB27099</t>
+        </is>
+      </c>
+      <c r="O44" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="P44" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="Q44" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R44" s="3" t="inlineStr"/>
+    </row>
+    <row r="45" ht="45" customHeight="1">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>c716bcad601a9d9ab8ce</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-18T03:56:25.967828+00:00</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-17T17:25:39+00:00</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr"/>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>- Hiring happens 1-6 months</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>Job / Hiring</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr"/>
+      <c r="H45" s="3" t="inlineStr"/>
+      <c r="I45" s="3" t="inlineStr"/>
+      <c r="J45" s="3" t="inlineStr"/>
+      <c r="K45" s="4" t="inlineStr">
+        <is>
+          <t>https://scontent-dfw6-2.cdninstagram.com/v/t51.82787-15/788924699_18087195047678962_4065300646317777670_n.heic?stp=dst-jpg_e35_sh2.08_tt6&amp;_nc_cat=109&amp;ig_cache_key=Mzk4ODMyOTQzNjcxNjUxMDE3Ng%3D%3D.3-ccb7-5&amp;ccb=7-5&amp;_nc_sid=58cdad&amp;efg=eyJ2ZW5jb2RlX3RhZyI6IlNUT1JZLnhwaWRzLjEwODAuc2RyLnJlZ3VsYXJfcGhvdG8uQzMifQ%3D%3D&amp;_nc_ohc=r1KisgbLBN0Q7kNvwGpdCaD&amp;_nc_oc=AdodVmaXg5vc8Ho_zZ3Mm8rqJD-iYH7jVBG7_BHU3uVxfw2beh9I0a5PTOS__-FZ_kQ&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=23&amp;se=7&amp;_nc_ht=scontent-dfw6-2.cdninstagram.com&amp;_nc_gid=eHz5TcyW0mp_pt15cJ6WDA&amp;_nc_ss=7e3ba&amp;oh=00_AQLwhQl2VA-wUB3JfXqeF5a1-Fs-FM7v5Cvk9dys3ot-KA&amp;oe=6AB29B46</t>
+        </is>
+      </c>
+      <c r="L45" s="4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/stories/zero2sudo/</t>
+        </is>
+      </c>
+      <c r="M45" s="3" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="N45" s="3" t="inlineStr">
+        <is>
+          <t>Hey Sudo, recap from the Tesla
+event at Chapel Hill:
+- Tailor your resume to the
+specific role, have similar
+keywords/skills/projects as they
+mention in the role
+- WHO method (What, How,
+Outcome)
+- Hiring happens 1-6 months
+before role start
+- Be yourself as much as possible
+in interviews
+- Referrals help, even from
+interns (goes to same place)
+- Best of the Best - why are you
+the best person that we should
+hire? (goes all the way up
+command chain)
+https://scontent-dfw6-2.cdninstagram.com/v/t51.82787-15/788924699_18087195047678962_4065300646317777670_n.heic?stp=dst-jpg_e35_sh2.08_tt6&amp;_nc_cat=109&amp;ig_cache_key=Mzk4ODMyOTQzNjcxNjUxMDE3Ng%3D%3D.3-ccb7-5&amp;ccb=7-5&amp;_nc_sid=58cdad&amp;efg=eyJ2ZW5jb2RlX3RhZyI6IlNUT1JZLnhwaWRzLjEwODAuc2RyLnJlZ3VsYXJfcGhvdG8uQzMifQ%3D%3D&amp;_nc_ohc=r1KisgbLBN0Q7kNvwGpdCaD&amp;_nc_oc=AdodVmaXg5vc8Ho_zZ3Mm8rqJD-iYH7jVBG7_BHU3uVxfw2beh9I0a5PTOS__-FZ_kQ&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=23&amp;se=7&amp;_nc_ht=scontent-dfw6-2.cdninstagram.com&amp;_nc_gid=eHz5TcyW0mp_pt15cJ6WDA&amp;_nc_ss=7e3ba&amp;oh=00_AQLwhQl2VA-wUB3JfXqeF5a1-Fs-FM7v5Cvk9dys3ot-KA&amp;oe=6AB29B46
+https://scontent-dfw6-2.cdninstagram.com/v/t51.82787-15/788924699_18087195047678962_4065300646317777670_n.heic?stp=dst-jpg_e35_s640x640_sh2.08_tt6&amp;_nc_cat=109&amp;ig_cache_key=Mzk4ODMyOTQzNjcxNjUxMDE3Ng%3D%3D.3-ccb7-5&amp;ccb=7-5&amp;_nc_sid=58cdad&amp;efg=eyJ2ZW5jb2RlX3RhZyI6IlNUT1JZLnhwaWRzLjEwODAuc2RyLnJlZ3VsYXJfcGhvdG8uQzMifQ%3D%3D&amp;_nc_ohc=r1KisgbLBN0Q7kNvwGpdCaD&amp;_nc_oc=AdodVmaXg5vc8Ho_zZ3Mm8rqJD-iYH7jVBG7_BHU3uVxfw2beh9I0a5PTOS__-FZ_kQ&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=23&amp;_nc_ht=scontent-dfw6-2.cdninstagram.com&amp;_nc_gid=eHz5TcyW0mp_pt15cJ6WDA&amp;_nc_ss=7e3ba&amp;oh=00_AQLDnG6D0On1tMrP5sUTsdtW39-tpQq7PkNZHeviJSdYUg&amp;oe=6AB29B46
+https://scontent-dfw5-2.cdninstagram.com/v/t51.2885-19/361942212_2508526442658147_3130876906989167533_n.jpg?stp=dst-jpg_e0_s150x150_tt6&amp;_nc_cat=100&amp;ig_cache_key=GMTMkhVjOYbTfekIAK0jkHT1G3MrbkULAAAB1501500j-ccb7-5&amp;ccb=7-5&amp;_nc_sid=669407&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDgwLkMzIn0%3D&amp;_nc_ohc=v_28DqPFYsAQ7kNvwEdRcyz&amp;_nc_oc=Adqw8M_x9B-a8shtOG5wRrb9an7G9olGpS9_wQd75NfCA1HGhLaideM0LC7_0tGzj_o&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=24&amp;_nc_ht=scontent-dfw5-2.cdninstagram.com&amp;_nc_ss=7e3ba&amp;oh=00_AQKjZ8LuZIyQWmMhzZRTIIXPovMdv5VlfhbUe2vSoVvRTA&amp;oe=6AB27099</t>
+        </is>
+      </c>
+      <c r="O45" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="P45" s="3" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="Q45" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R45" s="3" t="inlineStr"/>
+    </row>
+    <row r="46" ht="45" customHeight="1">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>d8f744b57e2f32c28c9b</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-18T03:56:28.030321+00:00</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-17T17:37:26+00:00</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>Google — webinar you posted JA, J,</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>New Grad / Early Career</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineering</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr"/>
+      <c r="I46" s="3" t="inlineStr"/>
+      <c r="J46" s="3" t="inlineStr"/>
+      <c r="K46" s="4" t="inlineStr">
+        <is>
+          <t>https://scontent-dfw5-2.cdninstagram.com/v/t51.82787-15/809209168_18087197012678962_1565929461932431535_n.heic?stp=dst-jpg_e35_sh2.08_tt6&amp;_nc_cat=100&amp;ig_cache_key=Mzk4ODMzNTM2NjgwNDgwMjc2MQ%3D%3D.3-ccb7-5&amp;ccb=7-5&amp;_nc_sid=58cdad&amp;efg=eyJ2ZW5jb2RlX3RhZyI6IlNUT1JZLnhwaWRzLjEwODAuc2RyLnJlZ3VsYXJfcGhvdG8uQzMifQ%3D%3D&amp;_nc_ohc=hyMuw1kltl4Q7kNvwGDmDfE&amp;_nc_oc=AdqP3Ta2dI1g0FVH7QyEE7uEOkgbBa3Q4hKWXs3n0cE6DhBALl74f1QRyALqnOSfz6A&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=23&amp;se=7&amp;_nc_ht=scontent-dfw5-2.cdninstagram.com&amp;_nc_gid=eHz5TcyW0mp_pt15cJ6WDA&amp;_nc_ss=7e3ba&amp;oh=00_AQIostWAzN_LeyMnpXj1RMvSP1_Q_e9HqHU6OvxXwXkAiA&amp;oe=6AB29612</t>
+        </is>
+      </c>
+      <c r="L46" s="4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/stories/zero2sudo/</t>
+        </is>
+      </c>
+      <c r="M46" s="3" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="N46" s="3" t="inlineStr">
+        <is>
+          <t>Google SWE New Grad RO!!!
+Got google return offer thank
+you for all you do for the cs
+students! Got my google
+interview last year because of a
+webinar you posted JA, J,
+| only know I'm matched to
+Youtube they said i won't be
+matched till 8 weeks b4 my start
+date
+https://scontent-dfw5-2.cdninstagram.com/v/t51.82787-15/809209168_18087197012678962_1565929461932431535_n.heic?stp=dst-jpg_e35_sh2.08_tt6&amp;_nc_cat=100&amp;ig_cache_key=Mzk4ODMzNTM2NjgwNDgwMjc2MQ%3D%3D.3-ccb7-5&amp;ccb=7-5&amp;_nc_sid=58cdad&amp;efg=eyJ2ZW5jb2RlX3RhZyI6IlNUT1JZLnhwaWRzLjEwODAuc2RyLnJlZ3VsYXJfcGhvdG8uQzMifQ%3D%3D&amp;_nc_ohc=hyMuw1kltl4Q7kNvwGDmDfE&amp;_nc_oc=AdqP3Ta2dI1g0FVH7QyEE7uEOkgbBa3Q4hKWXs3n0cE6DhBALl74f1QRyALqnOSfz6A&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=23&amp;se=7&amp;_nc_ht=scontent-dfw5-2.cdninstagram.com&amp;_nc_gid=eHz5TcyW0mp_pt15cJ6WDA&amp;_nc_ss=7e3ba&amp;oh=00_AQIostWAzN_LeyMnpXj1RMvSP1_Q_e9HqHU6OvxXwXkAiA&amp;oe=6AB29612
+https://scontent-dfw5-2.cdninstagram.com/v/t51.82787-15/809209168_18087197012678962_1565929461932431535_n.heic?stp=dst-jpg_e35_s640x640_sh2.08_tt6&amp;_nc_cat=100&amp;ig_cache_key=Mzk4ODMzNTM2NjgwNDgwMjc2MQ%3D%3D.3-ccb7-5&amp;ccb=7-5&amp;_nc_sid=58cdad&amp;efg=eyJ2ZW5jb2RlX3RhZyI6IlNUT1JZLnhwaWRzLjEwODAuc2RyLnJlZ3VsYXJfcGhvdG8uQzMifQ%3D%3D&amp;_nc_ohc=hyMuw1kltl4Q7kNvwGDmDfE&amp;_nc_oc=AdqP3Ta2dI1g0FVH7QyEE7uEOkgbBa3Q4hKWXs3n0cE6DhBALl74f1QRyALqnOSfz6A&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=23&amp;_nc_ht=scontent-dfw5-2.cdninstagram.com&amp;_nc_gid=eHz5TcyW0mp_pt15cJ6WDA&amp;_nc_ss=7e3ba&amp;oh=00_AQJzFWVHc5WeuM08e47_3LCv6Ija7-EHDaKsxGpsey7Cag&amp;oe=6AB29612
+https://scontent-dfw5-2.cdninstagram.com/v/t51.2885-19/361942212_2508526442658147_3130876906989167533_n.jpg?stp=dst-jpg_e0_s150x150_tt6&amp;_nc_cat=100&amp;ig_cache_key=GMTMkhVjOYbTfekIAK0jkHT1G3MrbkULAAAB1501500j-ccb7-5&amp;ccb=7-5&amp;_nc_sid=669407&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDgwLkMzIn0%3D&amp;_nc_ohc=v_28DqPFYsAQ7kNvwEdRcyz&amp;_nc_oc=Adqw8M_x9B-a8shtOG5wRrb9an7G9olGpS9_wQd75NfCA1HGhLaideM0LC7_0tGzj_o&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=24&amp;_nc_ht=scontent-dfw5-2.cdninstagram.com&amp;_nc_ss=7e3ba&amp;oh=00_AQKjZ8LuZIyQWmMhzZRTIIXPovMdv5VlfhbUe2vSoVvRTA&amp;oe=6AB27099</t>
+        </is>
+      </c>
+      <c r="O46" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="P46" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="Q46" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R46" s="3" t="inlineStr"/>
+    </row>
+    <row r="47" ht="45" customHeight="1">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>5ec01f615ec61f7238aa</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-18T03:56:45.854899+00:00</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-17T20:13:34+00:00</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>Adobe</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>Adobe — also no sign up form</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr"/>
+      <c r="H47" s="3" t="inlineStr"/>
+      <c r="I47" s="3" t="inlineStr"/>
+      <c r="J47" s="3" t="inlineStr"/>
+      <c r="K47" s="4" t="inlineStr">
+        <is>
+          <t>https://scontent-dfw6-1.cdninstagram.com/v/t51.82787-15/813976257_18087212606678962_600677638285630895_n.heic?stp=dst-jpg_e35_sh2.08_tt6&amp;_nc_cat=101&amp;ig_cache_key=Mzk4ODQxMzk1MjcwNjYxNTUwMA%3D%3D.3-ccb7-5&amp;ccb=7-5&amp;_nc_sid=58cdad&amp;efg=eyJ2ZW5jb2RlX3RhZyI6IlNUT1JZLnhwaWRzLjEwODAuc2RyLnJlZ3VsYXJfcGhvdG8uQzMifQ%3D%3D&amp;_nc_ohc=mB7SsEg8mAcQ7kNvwH7ifI4&amp;_nc_oc=AdrgaQy7PBD-5nGixGfL9Zm9M9qCO-UwaBNx4BPlBGPKDnHMEuxIZR6RGEskG80WK3M&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=23&amp;se=7&amp;_nc_ht=scontent-dfw6-1.cdninstagram.com&amp;_nc_gid=eHz5TcyW0mp_pt15cJ6WDA&amp;_nc_ss=7e3ba&amp;oh=00_AQLcplPJMSsGcX-eInoBlbJjbtdXSHaxWs8IMJ0bNGTzjw&amp;oe=6AB27AB6</t>
+        </is>
+      </c>
+      <c r="L47" s="4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/stories/zero2sudo/</t>
+        </is>
+      </c>
+      <c r="M47" s="3" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="N47" s="3" t="inlineStr">
+        <is>
+          <t>Adobe Intern
+@ rolling bests)!
+epee matters more than referrals
+aa tor Adobe!
+in the adobe event they also said
+that referrals matter but speed
+matters more and for ai they said
+that they are only gonna use it in
+a few questions and not for all in
+the interviews and she said that
+they are gonna wrap up their
+hiring around march
+| wasn’t there for the first 20ish
+minutes for the event so idk what
+happened there but there was
+also no sign up form
+she also said that they don’t use
+Al to look through candidates
+https://scontent-dfw6-1.cdninstagram.com/v/t51.82787-15/813976257_18087212606678962_600677638285630895_n.heic?stp=dst-jpg_e35_sh2.08_tt6&amp;_nc_cat=101&amp;ig_cache_key=Mzk4ODQxMzk1MjcwNjYxNTUwMA%3D%3D.3-ccb7-5&amp;ccb=7-5&amp;_nc_sid=58cdad&amp;efg=eyJ2ZW5jb2RlX3RhZyI6IlNUT1JZLnhwaWRzLjEwODAuc2RyLnJlZ3VsYXJfcGhvdG8uQzMifQ%3D%3D&amp;_nc_ohc=mB7SsEg8mAcQ7kNvwH7ifI4&amp;_nc_oc=AdrgaQy7PBD-5nGixGfL9Zm9M9qCO-UwaBNx4BPlBGPKDnHMEuxIZR6RGEskG80WK3M&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=23&amp;se=7&amp;_nc_ht=scontent-dfw6-1.cdninstagram.com&amp;_nc_gid=eHz5TcyW0mp_pt15cJ6WDA&amp;_nc_ss=7e3ba&amp;oh=00_AQLcplPJMSsGcX-eInoBlbJjbtdXSHaxWs8IMJ0bNGTzjw&amp;oe=6AB27AB6
+https://scontent-dfw6-1.cdninstagram.com/v/t51.82787-15/813976257_18087212606678962_600677638285630895_n.heic?stp=dst-jpg_e35_s640x640_sh2.08_tt6&amp;_nc_cat=101&amp;ig_cache_key=Mzk4ODQxMzk1MjcwNjYxNTUwMA%3D%3D.3-ccb7-5&amp;ccb=7-5&amp;_nc_sid=58cdad&amp;efg=eyJ2ZW5jb2RlX3RhZyI6IlNUT1JZLnhwaWRzLjEwODAuc2RyLnJlZ3VsYXJfcGhvdG8uQzMifQ%3D%3D&amp;_nc_ohc=mB7SsEg8mAcQ7kNvwH7ifI4&amp;_nc_oc=AdrgaQy7PBD-5nGixGfL9Zm9M9qCO-UwaBNx4BPlBGPKDnHMEuxIZR6RGEskG80WK3M&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=23&amp;_nc_ht=scontent-dfw6-1.cdninstagram.com&amp;_nc_gid=eHz5TcyW0mp_pt15cJ6WDA&amp;_nc_ss=7e3ba&amp;oh=00_AQJmDHRanLsPRRuz018MKNgajUmLnPE_BRNLe2hAqyiJ5Q&amp;oe=6AB27AB6
+https://scontent-dfw5-2.cdninstagram.com/v/t51.2885-19/361942212_2508526442658147_3130876906989167533_n.jpg?stp=dst-jpg_e0_s150x150_tt6&amp;_nc_cat=100&amp;ig_cache_key=GMTMkhVjOYbTfekIAK0jkHT1G3MrbkULAAAB1501500j-ccb7-5&amp;ccb=7-5&amp;_nc_sid=669407&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDgwLkMzIn0%3D&amp;_nc_ohc=v_28DqPFYsAQ7kNvwEdRcyz&amp;_nc_oc=Adqw8M_x9B-a8shtOG5wRrb9an7G9olGpS9_wQd75NfCA1HGhLaideM0LC7_0tGzj_o&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=24&amp;_nc_ht=scontent-dfw5-2.cdninstagram.com&amp;_nc_ss=7e3ba&amp;oh=00_AQKjZ8LuZIyQWmMhzZRTIIXPovMdv5VlfhbUe2vSoVvRTA&amp;oe=6AB27099</t>
+        </is>
+      </c>
+      <c r="O47" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="P47" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="Q47" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R47" s="3" t="inlineStr"/>
+    </row>
+    <row r="48" ht="45" customHeight="1">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>406eecd407d7e310c1bb</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-18T03:56:54.958591+00:00</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-17T20:35:03+00:00</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr"/>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>So many Capi SWE Intern Offers!</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineering</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr"/>
+      <c r="I48" s="3" t="inlineStr"/>
+      <c r="J48" s="3" t="inlineStr"/>
+      <c r="K48" s="4" t="inlineStr">
+        <is>
+          <t>https://scontent-dfw6-1.cdninstagram.com/v/t51.82787-15/814768840_18087214964678962_300587807414299988_n.heic?stp=dst-jpg_e35_sh2.08_tt6&amp;_nc_cat=102&amp;ig_cache_key=Mzk4ODQyNDc2MjY2MTAyNzcwOA%3D%3D.3-ccb7-5&amp;ccb=7-5&amp;_nc_sid=58cdad&amp;efg=eyJ2ZW5jb2RlX3RhZyI6IlNUT1JZLnhwaWRzLjEwODAuc2RyLnJlZ3VsYXJfcGhvdG8uQzMifQ%3D%3D&amp;_nc_ohc=pKt1LD4ViCkQ7kNvwGmc1Xt&amp;_nc_oc=AdoWWXXPfejqt7fr8TqU4wiOJQL5Kapkkj3oZVJYjGdMXzvek1-BVeQqoMxaOTP3aSw&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=23&amp;se=7&amp;_nc_ht=scontent-dfw6-1.cdninstagram.com&amp;_nc_gid=eHz5TcyW0mp_pt15cJ6WDA&amp;_nc_ss=7e3ba&amp;oh=00_AQLfVG2TXYuw4-wQ30d9xFs07gxCXJmKpbd9Zr-A8UPhHQ&amp;oe=6AB28EC4</t>
+        </is>
+      </c>
+      <c r="L48" s="4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/stories/zero2sudo/</t>
+        </is>
+      </c>
+      <c r="M48" s="3" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="N48" s="3" t="inlineStr">
+        <is>
+          <t>Replied to your story
+got c1tip as well, helpful info on
+the ai assist ty. litearlly heard
+back in less than 24 hours as well
+So many Capi SWE Intern Offers!
+https://scontent-dfw6-1.cdninstagram.com/v/t51.82787-15/814768840_18087214964678962_300587807414299988_n.heic?stp=dst-jpg_e35_sh2.08_tt6&amp;_nc_cat=102&amp;ig_cache_key=Mzk4ODQyNDc2MjY2MTAyNzcwOA%3D%3D.3-ccb7-5&amp;ccb=7-5&amp;_nc_sid=58cdad&amp;efg=eyJ2ZW5jb2RlX3RhZyI6IlNUT1JZLnhwaWRzLjEwODAuc2RyLnJlZ3VsYXJfcGhvdG8uQzMifQ%3D%3D&amp;_nc_ohc=pKt1LD4ViCkQ7kNvwGmc1Xt&amp;_nc_oc=AdoWWXXPfejqt7fr8TqU4wiOJQL5Kapkkj3oZVJYjGdMXzvek1-BVeQqoMxaOTP3aSw&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=23&amp;se=7&amp;_nc_ht=scontent-dfw6-1.cdninstagram.com&amp;_nc_gid=eHz5TcyW0mp_pt15cJ6WDA&amp;_nc_ss=7e3ba&amp;oh=00_AQLfVG2TXYuw4-wQ30d9xFs07gxCXJmKpbd9Zr-A8UPhHQ&amp;oe=6AB28EC4
+https://scontent-dfw6-1.cdninstagram.com/v/t51.82787-15/814768840_18087214964678962_300587807414299988_n.heic?stp=dst-jpg_e35_s640x640_sh2.08_tt6&amp;_nc_cat=102&amp;ig_cache_key=Mzk4ODQyNDc2MjY2MTAyNzcwOA%3D%3D.3-ccb7-5&amp;ccb=7-5&amp;_nc_sid=58cdad&amp;efg=eyJ2ZW5jb2RlX3RhZyI6IlNUT1JZLnhwaWRzLjEwODAuc2RyLnJlZ3VsYXJfcGhvdG8uQzMifQ%3D%3D&amp;_nc_ohc=pKt1LD4ViCkQ7kNvwGmc1Xt&amp;_nc_oc=AdoWWXXPfejqt7fr8TqU4wiOJQL5Kapkkj3oZVJYjGdMXzvek1-BVeQqoMxaOTP3aSw&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=23&amp;_nc_ht=scontent-dfw6-1.cdninstagram.com&amp;_nc_gid=eHz5TcyW0mp_pt15cJ6WDA&amp;_nc_ss=7e3ba&amp;oh=00_AQKK9OBBGgHLdlREGZEWhyBfKCkjYAZhPcMzTH2etxQsrg&amp;oe=6AB28EC4
+https://scontent-dfw5-2.cdninstagram.com/v/t51.2885-19/361942212_2508526442658147_3130876906989167533_n.jpg?stp=dst-jpg_e0_s150x150_tt6&amp;_nc_cat=100&amp;ig_cache_key=GMTMkhVjOYbTfekIAK0jkHT1G3MrbkULAAAB1501500j-ccb7-5&amp;ccb=7-5&amp;_nc_sid=669407&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDgwLkMzIn0%3D&amp;_nc_ohc=v_28DqPFYsAQ7kNvwEdRcyz&amp;_nc_oc=Adqw8M_x9B-a8shtOG5wRrb9an7G9olGpS9_wQd75NfCA1HGhLaideM0LC7_0tGzj_o&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=24&amp;_nc_ht=scontent-dfw5-2.cdninstagram.com&amp;_nc_ss=7e3ba&amp;oh=00_AQKjZ8LuZIyQWmMhzZRTIIXPovMdv5VlfhbUe2vSoVvRTA&amp;oe=6AB27099</t>
+        </is>
+      </c>
+      <c r="O48" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="P48" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="Q48" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R48" s="3" t="inlineStr"/>
+    </row>
+    <row r="49" ht="45" customHeight="1">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>a99c75e25c9a557a5480</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-18T03:57:00.309434+00:00</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-17T21:45:38+00:00</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr"/>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>This is why | care so much about making opportunity</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr"/>
+      <c r="H49" s="3" t="inlineStr"/>
+      <c r="I49" s="3" t="inlineStr"/>
+      <c r="J49" s="3" t="inlineStr"/>
+      <c r="K49" s="4" t="inlineStr">
+        <is>
+          <t>https://scontent-dfw5-1.cdninstagram.com/v/t51.82787-15/814695558_18087220370678962_7673257959919455186_n.heic?stp=dst-jpg_e35_sh2.08_tt6&amp;_nc_cat=105&amp;ig_cache_key=Mzk4ODQ2MDI4NjYyNDg0MzIxMQ%3D%3D.3-ccb7-5&amp;ccb=7-5&amp;_nc_sid=58cdad&amp;efg=eyJ2ZW5jb2RlX3RhZyI6IlNUT1JZLnhwaWRzLjEwODAuc2RyLnJlZ3VsYXJfcGhvdG8uQzMifQ%3D%3D&amp;_nc_ohc=cjWX3Z2jFwgQ7kNvwFQwL12&amp;_nc_oc=AdpT1A9Oi-S9coUbMd4aNFpXGgvavHvrRTkuWPbPVSiVxtBpWJNvyhWFrgSD_wWpd1k&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=23&amp;se=7&amp;_nc_ht=scontent-dfw5-1.cdninstagram.com&amp;_nc_gid=eHz5TcyW0mp_pt15cJ6WDA&amp;_nc_ss=7e3ba&amp;oh=00_AQLt2FiRSa8REgSoEbK6HJbEM2xWYlfJE05brCM6MV0KZg&amp;oe=6AB299D1</t>
+        </is>
+      </c>
+      <c r="L49" s="4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/stories/zero2sudo/</t>
+        </is>
+      </c>
+      <c r="M49" s="3" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="N49" s="3" t="inlineStr">
+        <is>
+          <t>So many non-target students made it to Bloomberg
+last year and crushed it. Never let anyone tell you
+what you deserve (unless it’s better than you
+expect), and never let where you start determine
+where you finish.
+This is why | care so much about making opportunity
+more accessible :)
+Same A, if you scroll up in
+our chat you can see | got
+headcounted initially, but
+persistence paid off
+Thanks for everything you do!
+| applied through your link last
+year.
+ae
+I'm the first ever intern at bb
+from my university purely
+because of your stories &amp;
+ae
+lets fkn go! it's super funny bc
+gatekeepers tried claiming
+people would be blacklisted for
+applying. in reality, multiple
+companies confirmed with us
+last year that they just want to
+hire competent candidates.
+good people exist anywhere,
+companies don't care about
+people "trying harder" to find an
+event link or some dumbass shit
+like that &amp; great job man :)
+https://scontent-dfw5-1.cdninstagram.com/v/t51.82787-15/814695558_18087220370678962_7673257959919455186_n.heic?stp=dst-jpg_e35_sh2.08_tt6&amp;_nc_cat=105&amp;ig_cache_key=Mzk4ODQ2MDI4NjYyNDg0MzIxMQ%3D%3D.3-ccb7-5&amp;ccb=7-5&amp;_nc_sid=58cdad&amp;efg=eyJ2ZW5jb2RlX3RhZyI6IlNUT1JZLnhwaWRzLjEwODAuc2RyLnJlZ3VsYXJfcGhvdG8uQzMifQ%3D%3D&amp;_nc_ohc=cjWX3Z2jFwgQ7kNvwFQwL12&amp;_nc_oc=AdpT1A9Oi-S9coUbMd4aNFpXGgvavHvrRTkuWPbPVSiVxtBpWJNvyhWFrgSD_wWpd1k&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=23&amp;se=7&amp;_nc_ht=scontent-dfw5-1.cdninstagram.com&amp;_nc_gid=eHz5TcyW0mp_pt15cJ6WDA&amp;_nc_ss=7e3ba&amp;oh=00_AQLt2FiRSa8REgSoEbK6HJbEM2xWYlfJE05brCM6MV0KZg&amp;oe=6AB299D1
+https://scontent-dfw5-1.cdninstagram.com/v/t51.82787-15/814695558_18087220370678962_7673257959919455186_n.heic?stp=dst-jpg_e35_s640x640_sh2.08_tt6&amp;_nc_cat=105&amp;ig_cache_key=Mzk4ODQ2MDI4NjYyNDg0MzIxMQ%3D%3D.3-ccb7-5&amp;ccb=7-5&amp;_nc_sid=58cdad&amp;efg=eyJ2ZW5jb2RlX3RhZyI6IlNUT1JZLnhwaWRzLjEwODAuc2RyLnJlZ3VsYXJfcGhvdG8uQzMifQ%3D%3D&amp;_nc_ohc=cjWX3Z2jFwgQ7kNvwFQwL12&amp;_nc_oc=AdpT1A9Oi-S9coUbMd4aNFpXGgvavHvrRTkuWPbPVSiVxtBpWJNvyhWFrgSD_wWpd1k&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=23&amp;_nc_ht=scontent-dfw5-1.cdninstagram.com&amp;_nc_gid=eHz5TcyW0mp_pt15cJ6WDA&amp;_nc_ss=7e3ba&amp;oh=00_AQKv6hKoYDUUuRWKaovEu-W_i3fy911SUhhyKWdW3GqDGw&amp;oe=6AB299D1
+https://scontent-dfw5-2.cdninstagram.com/v/t51.2885-19/361942212_2508526442658147_3130876906989167533_n.jpg?stp=dst-jpg_e0_s150x150_tt6&amp;_nc_cat=100&amp;ig_cache_key=GMTMkhVjOYbTfekIAK0jkHT1G3MrbkULAAAB1501500j-ccb7-5&amp;ccb=7-5&amp;_nc_sid=669407&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDgwLkMzIn0%3D&amp;_nc_ohc=v_28DqPFYsAQ7kNvwEdRcyz&amp;_nc_oc=Adqw8M_x9B-a8shtOG5wRrb9an7G9olGpS9_wQd75NfCA1HGhLaideM0LC7_0tGzj_o&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=24&amp;_nc_ht=scontent-dfw5-2.cdninstagram.com&amp;_nc_ss=7e3ba&amp;oh=00_AQKjZ8LuZIyQWmMhzZRTIIXPovMdv5VlfhbUe2vSoVvRTA&amp;oe=6AB27099</t>
+        </is>
+      </c>
+      <c r="O49" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="P49" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="Q49" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R49" s="3" t="inlineStr"/>
+    </row>
+    <row r="50" ht="45" customHeight="1">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>b05a980a5e5c08b9287d</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-18T03:57:03.026869+00:00</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-17T21:49:10+00:00</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr"/>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>career fair but we are definitely</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>Recruiting / Career Event</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr"/>
+      <c r="H50" s="3" t="inlineStr"/>
+      <c r="I50" s="3" t="inlineStr"/>
+      <c r="J50" s="3" t="inlineStr"/>
+      <c r="K50" s="4" t="inlineStr">
+        <is>
+          <t>https://scontent-dfw5-1.cdninstagram.com/v/t51.82787-15/814229705_18087220610678962_85839488440364683_n.heic?stp=dst-jpg_e35_sh2.08_tt6&amp;_nc_cat=105&amp;ig_cache_key=Mzk4ODQ2MjA2ODY5MjM1ODkwOQ%3D%3D.3-ccb7-5&amp;ccb=7-5&amp;_nc_sid=58cdad&amp;efg=eyJ2ZW5jb2RlX3RhZyI6IlNUT1JZLnhwaWRzLjEwODAuc2RyLnJlZ3VsYXJfcGhvdG8uQzMifQ%3D%3D&amp;_nc_ohc=8_nKWHMwEBkQ7kNvwFHtp7M&amp;_nc_oc=Adq8Vb2DwR7WFk4raII5dwO7zqnLZ11FjpaSySsL8C1v09BNzAjMd-OvEozUUr_GoqU&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=23&amp;se=7&amp;_nc_ht=scontent-dfw5-1.cdninstagram.com&amp;_nc_gid=eHz5TcyW0mp_pt15cJ6WDA&amp;_nc_ss=7e3ba&amp;oh=00_AQJ0BfSD_GObVyneapxWhUFOmU8UAUXpUBpFC670fF8FPg&amp;oe=6AB2850B</t>
+        </is>
+      </c>
+      <c r="L50" s="4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/stories/zero2sudo/</t>
+        </is>
+      </c>
+      <c r="M50" s="3" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="N50" s="3" t="inlineStr">
+        <is>
+          <t>ARM recruiter clarification on
+application consideration!
+Hey hey, someone flagged
+this for me, this is probably a
+misunderstanding from the
+career fair but we are definitely
+still considering applications
+from our original application
+window being open. We are
+no longer accepting new
+applications outside of career
+fair signups, that could be the
+confusion point from the fair.
+https://scontent-dfw5-1.cdninstagram.com/v/t51.82787-15/814229705_18087220610678962_85839488440364683_n.heic?stp=dst-jpg_e35_sh2.08_tt6&amp;_nc_cat=105&amp;ig_cache_key=Mzk4ODQ2MjA2ODY5MjM1ODkwOQ%3D%3D.3-ccb7-5&amp;ccb=7-5&amp;_nc_sid=58cdad&amp;efg=eyJ2ZW5jb2RlX3RhZyI6IlNUT1JZLnhwaWRzLjEwODAuc2RyLnJlZ3VsYXJfcGhvdG8uQzMifQ%3D%3D&amp;_nc_ohc=8_nKWHMwEBkQ7kNvwFHtp7M&amp;_nc_oc=Adq8Vb2DwR7WFk4raII5dwO7zqnLZ11FjpaSySsL8C1v09BNzAjMd-OvEozUUr_GoqU&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=23&amp;se=7&amp;_nc_ht=scontent-dfw5-1.cdninstagram.com&amp;_nc_gid=eHz5TcyW0mp_pt15cJ6WDA&amp;_nc_ss=7e3ba&amp;oh=00_AQJ0BfSD_GObVyneapxWhUFOmU8UAUXpUBpFC670fF8FPg&amp;oe=6AB2850B
+https://scontent-dfw5-1.cdninstagram.com/v/t51.82787-15/814229705_18087220610678962_85839488440364683_n.heic?stp=dst-jpg_e35_s640x640_sh2.08_tt6&amp;_nc_cat=105&amp;ig_cache_key=Mzk4ODQ2MjA2ODY5MjM1ODkwOQ%3D%3D.3-ccb7-5&amp;ccb=7-5&amp;_nc_sid=58cdad&amp;efg=eyJ2ZW5jb2RlX3RhZyI6IlNUT1JZLnhwaWRzLjEwODAuc2RyLnJlZ3VsYXJfcGhvdG8uQzMifQ%3D%3D&amp;_nc_ohc=8_nKWHMwEBkQ7kNvwFHtp7M&amp;_nc_oc=Adq8Vb2DwR7WFk4raII5dwO7zqnLZ11FjpaSySsL8C1v09BNzAjMd-OvEozUUr_GoqU&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=23&amp;_nc_ht=scontent-dfw5-1.cdninstagram.com&amp;_nc_gid=eHz5TcyW0mp_pt15cJ6WDA&amp;_nc_ss=7e3ba&amp;oh=00_AQIBe2RX7D6PQfZ5GpMe85mCb3lbJ-gRAPPbE_xN3rABGA&amp;oe=6AB2850B
+https://scontent-dfw5-2.cdninstagram.com/v/t51.2885-19/361942212_2508526442658147_3130876906989167533_n.jpg?stp=dst-jpg_e0_s150x150_tt6&amp;_nc_cat=100&amp;ig_cache_key=GMTMkhVjOYbTfekIAK0jkHT1G3MrbkULAAAB1501500j-ccb7-5&amp;ccb=7-5&amp;_nc_sid=669407&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDgwLkMzIn0%3D&amp;_nc_ohc=v_28DqPFYsAQ7kNvwEdRcyz&amp;_nc_oc=Adqw8M_x9B-a8shtOG5wRrb9an7G9olGpS9_wQd75NfCA1HGhLaideM0LC7_0tGzj_o&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=24&amp;_nc_ht=scontent-dfw5-2.cdninstagram.com&amp;_nc_ss=7e3ba&amp;oh=00_AQKjZ8LuZIyQWmMhzZRTIIXPovMdv5VlfhbUe2vSoVvRTA&amp;oe=6AB27099</t>
+        </is>
+      </c>
+      <c r="O50" s="3" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="P50" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="Q50" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R50" s="3" t="inlineStr"/>
+    </row>
+    <row r="51" ht="45" customHeight="1">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>cb892eb20bb5e8bf02de</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-18T03:57:42.780142+00:00</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-17T23:38:08+00:00</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>Amazon — 1AZ0N SWE INTERN 2027 &amp;</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineering</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="I51" s="3" t="inlineStr"/>
+      <c r="J51" s="3" t="inlineStr"/>
+      <c r="K51" s="4" t="inlineStr">
+        <is>
+          <t>https://scontent-dfw6-1.cdninstagram.com/v/t51.82787-15/814779823_18087230822678962_7861859619461180195_n.heic?stp=dst-jpg_e35_sh2.08_tt6&amp;_nc_cat=103&amp;ig_cache_key=Mzk4ODUxNjkwOTI4NjA1MTY1Ng%3D%3D.3-ccb7-5&amp;ccb=7-5&amp;_nc_sid=58cdad&amp;efg=eyJ2ZW5jb2RlX3RhZyI6IlNUT1JZLnhwaWRzLjEwODAuc2RyLnJlZ3VsYXJfcGhvdG8uQzMifQ%3D%3D&amp;_nc_ohc=K22FdASUScsQ7kNvwEvHaFi&amp;_nc_oc=AdoQIek4FQMqLlmJYPzidfEr7oCV4F82zJCRax858_LfrkYKuBPCI8uXwqX7MkpngfU&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=23&amp;se=7&amp;_nc_ht=scontent-dfw6-1.cdninstagram.com&amp;_nc_gid=eHz5TcyW0mp_pt15cJ6WDA&amp;_nc_ss=7e3ba&amp;oh=00_AQJni_oy7mNWkib4ab3OL8yIdviP21Y9xzY-Z58nUm0O7g&amp;oe=6AB28C0F</t>
+        </is>
+      </c>
+      <c r="L51" s="4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/stories/zero2sudo/</t>
+        </is>
+      </c>
+      <c r="M51" s="3" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="N51" s="3" t="inlineStr">
+        <is>
+          <t>Replied to your story
+Ask your Amazon questions!
+2027 (USA)
+Type something...
+1AZ0N SWE INTERN 2027 &amp;
+HUGE DROP @ @ @ gal
+interning at amazon rn Imk if | can
+provide any helpful info abt the
+process
+| think at this point you probbaly
+have heard it so many times but
+Leadership Principles are so so
+so important i think it helps to
+literally sit down and study them
+yessir! ty for sharing A.A.
+https://scontent-dfw6-1.cdninstagram.com/v/t51.82787-15/814779823_18087230822678962_7861859619461180195_n.heic?stp=dst-jpg_e35_sh2.08_tt6&amp;_nc_cat=103&amp;ig_cache_key=Mzk4ODUxNjkwOTI4NjA1MTY1Ng%3D%3D.3-ccb7-5&amp;ccb=7-5&amp;_nc_sid=58cdad&amp;efg=eyJ2ZW5jb2RlX3RhZyI6IlNUT1JZLnhwaWRzLjEwODAuc2RyLnJlZ3VsYXJfcGhvdG8uQzMifQ%3D%3D&amp;_nc_ohc=K22FdASUScsQ7kNvwEvHaFi&amp;_nc_oc=AdoQIek4FQMqLlmJYPzidfEr7oCV4F82zJCRax858_LfrkYKuBPCI8uXwqX7MkpngfU&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=23&amp;se=7&amp;_nc_ht=scontent-dfw6-1.cdninstagram.com&amp;_nc_gid=eHz5TcyW0mp_pt15cJ6WDA&amp;_nc_ss=7e3ba&amp;oh=00_AQJni_oy7mNWkib4ab3OL8yIdviP21Y9xzY-Z58nUm0O7g&amp;oe=6AB28C0F
+https://scontent-dfw6-1.cdninstagram.com/v/t51.82787-15/814779823_18087230822678962_7861859619461180195_n.heic?stp=dst-jpg_e35_s640x640_sh2.08_tt6&amp;_nc_cat=103&amp;ig_cache_key=Mzk4ODUxNjkwOTI4NjA1MTY1Ng%3D%3D.3-ccb7-5&amp;ccb=7-5&amp;_nc_sid=58cdad&amp;efg=eyJ2ZW5jb2RlX3RhZyI6IlNUT1JZLnhwaWRzLjEwODAuc2RyLnJlZ3VsYXJfcGhvdG8uQzMifQ%3D%3D&amp;_nc_ohc=K22FdASUScsQ7kNvwEvHaFi&amp;_nc_oc=AdoQIek4FQMqLlmJYPzidfEr7oCV4F82zJCRax858_LfrkYKuBPCI8uXwqX7MkpngfU&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=23&amp;_nc_ht=scontent-dfw6-1.cdninstagram.com&amp;_nc_gid=eHz5TcyW0mp_pt15cJ6WDA&amp;_nc_ss=7e3ba&amp;oh=00_AQI_SnA4LGBN9T2S09E-BZmktP92CboF4vixfqJC0UiyTA&amp;oe=6AB28C0F
+https://scontent-dfw5-2.cdninstagram.com/v/t51.2885-19/361942212_2508526442658147_3130876906989167533_n.jpg?stp=dst-jpg_e0_s150x150_tt6&amp;_nc_cat=100&amp;ig_cache_key=GMTMkhVjOYbTfekIAK0jkHT1G3MrbkULAAAB1501500j-ccb7-5&amp;ccb=7-5&amp;_nc_sid=669407&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDgwLkMzIn0%3D&amp;_nc_ohc=v_28DqPFYsAQ7kNvwEdRcyz&amp;_nc_oc=Adqw8M_x9B-a8shtOG5wRrb9an7G9olGpS9_wQd75NfCA1HGhLaideM0LC7_0tGzj_o&amp;_nc_ad=z-m&amp;_nc_cid=0&amp;_nc_zt=24&amp;_nc_ht=scontent-dfw5-2.cdninstagram.com&amp;_nc_ss=7e3ba&amp;oh=00_AQKjZ8LuZIyQWmMhzZRTIIXPovMdv5VlfhbUe2vSoVvRTA&amp;oe=6AB27099</t>
+        </is>
+      </c>
+      <c r="O51" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="P51" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="Q51" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R51" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:R41"/>
+  <autoFilter ref="A1:R51"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId2"/>
@@ -4436,6 +5335,26 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L40" r:id="rId78"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K41" r:id="rId79"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K42" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L42" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K43" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L43" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K44" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L44" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K45" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L45" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K46" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L46" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K47" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L47" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K48" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L48" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K49" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L49" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K50" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L50" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K51" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L51" r:id="rId100"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>